<commit_message>
3.53.0: the old log book also as a PDF / photo read by the AI, the names the AI finds (ticked), the lines to look at, the duplicates listed, the format (Excel)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XSqYFVL6aBM3vhiHD4bnxW
</commit_message>
<xml_diff>
--- a/test/fixtures/sheets/maint_logbook.xlsx
+++ b/test/fixtures/sheets/maint_logbook.xlsx
@@ -836,7 +836,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -962,9 +962,47 @@
         <v>1416</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6">
+        <v>3</v>
+      </c>
+      <c r="B6" t="str">
+        <v/>
+      </c>
+      <c r="C6" t="str">
+        <v/>
+      </c>
+      <c r="D6" t="str">
+        <v/>
+      </c>
+      <c r="E6" t="str">
+        <v>Coolant</v>
+      </c>
+      <c r="F6">
+        <v>2</v>
+      </c>
+      <c r="G6" t="str">
+        <v>Ltr</v>
+      </c>
+      <c r="H6">
+        <v>250</v>
+      </c>
+      <c r="I6">
+        <v>450</v>
+      </c>
+      <c r="J6">
+        <v>81</v>
+      </c>
+      <c r="K6">
+        <v>541</v>
+      </c>
+      <c r="L6">
+        <v>541</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L6"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>